<commit_message>
Actualizar motores y catálogo visual
</commit_message>
<xml_diff>
--- a/Control_Fotos_CodeBrew.xlsx
+++ b/Control_Fotos_CodeBrew.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Control de fotos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Control de fotos'!$A$7:$I$992</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Control de fotos'!$A$7:$I$997</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -220,8 +220,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ControlFotosCodigoDia" displayName="ControlFotosCodigoDia" ref="A7:I992" headerRowCount="1">
-  <autoFilter ref="A7:I992"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ControlFotosCodigoDia" displayName="ControlFotosCodigoDia" ref="A7:I997" headerRowCount="1">
+  <autoFilter ref="A7:I997"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ESTADO FOTO"/>
     <tableColumn id="2" name="CÓDIGO DÍA"/>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I992"/>
+  <dimension ref="A1:I997"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -575,17 +575,17 @@
     </row>
     <row r="4">
       <c r="A4" s="3">
-        <f>COUNTA(B8:B992)</f>
+        <f>COUNTA(B8:B997)</f>
         <v/>
       </c>
       <c r="B4" s="3" t="n"/>
       <c r="C4" s="3">
-        <f>COUNTIF(A8:A992,"CON FOTO")</f>
+        <f>COUNTIF(A8:A997,"CON FOTO")</f>
         <v/>
       </c>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3">
-        <f>COUNTIF(A8:A992,"FALTA FOTO")</f>
+        <f>COUNTIF(A8:A997,"FALTA FOTO")</f>
         <v/>
       </c>
       <c r="F4" s="3" t="n"/>
@@ -29306,17 +29306,17 @@
       </c>
       <c r="B827" s="7" t="inlineStr">
         <is>
-          <t>16531</t>
+          <t>16540</t>
         </is>
       </c>
       <c r="C827" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11174779</t>
         </is>
       </c>
       <c r="D827" t="inlineStr">
         <is>
-          <t>Sp26NEBlack</t>
+          <t>Wt26CCGl16Red</t>
         </is>
       </c>
       <c r="E827" t="inlineStr">
@@ -29341,17 +29341,17 @@
       </c>
       <c r="B828" s="7" t="inlineStr">
         <is>
-          <t>16532</t>
+          <t>16541</t>
         </is>
       </c>
       <c r="C828" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11174804</t>
         </is>
       </c>
       <c r="D828" t="inlineStr">
         <is>
-          <t>Sp26NECrossB</t>
+          <t>Wt26BTLStanley</t>
         </is>
       </c>
       <c r="E828" t="inlineStr">
@@ -29376,17 +29376,17 @@
       </c>
       <c r="B829" s="7" t="inlineStr">
         <is>
-          <t>16540</t>
+          <t>16543</t>
         </is>
       </c>
       <c r="C829" s="7" t="inlineStr">
         <is>
-          <t>11174779</t>
+          <t>11174795</t>
         </is>
       </c>
       <c r="D829" t="inlineStr">
         <is>
-          <t>Wt26CCGl16Red</t>
+          <t>Wt26CC24Spinner</t>
         </is>
       </c>
       <c r="E829" t="inlineStr">
@@ -29411,17 +29411,17 @@
       </c>
       <c r="B830" s="7" t="inlineStr">
         <is>
-          <t>16541</t>
+          <t>16544</t>
         </is>
       </c>
       <c r="C830" s="7" t="inlineStr">
         <is>
-          <t>11174804</t>
+          <t>11177277</t>
         </is>
       </c>
       <c r="D830" t="inlineStr">
         <is>
-          <t>Wt26BTLStanley</t>
+          <t>Wt26CC24Choco</t>
         </is>
       </c>
       <c r="E830" t="inlineStr">
@@ -29446,17 +29446,17 @@
       </c>
       <c r="B831" s="7" t="inlineStr">
         <is>
-          <t>16543</t>
+          <t>16545</t>
         </is>
       </c>
       <c r="C831" s="7" t="inlineStr">
         <is>
-          <t>11174795</t>
+          <t>11174808</t>
         </is>
       </c>
       <c r="D831" t="inlineStr">
         <is>
-          <t>Wt26CC24Spinner</t>
+          <t>Wt26SSCC24Grad</t>
         </is>
       </c>
       <c r="E831" t="inlineStr">
@@ -29481,17 +29481,17 @@
       </c>
       <c r="B832" s="7" t="inlineStr">
         <is>
-          <t>16544</t>
+          <t>16546</t>
         </is>
       </c>
       <c r="C832" s="7" t="inlineStr">
         <is>
-          <t>11177277</t>
+          <t>11174811</t>
         </is>
       </c>
       <c r="D832" t="inlineStr">
         <is>
-          <t>Wt26CC24Choco</t>
+          <t>Wt26SS30Jac</t>
         </is>
       </c>
       <c r="E832" t="inlineStr">
@@ -29516,17 +29516,17 @@
       </c>
       <c r="B833" s="7" t="inlineStr">
         <is>
-          <t>16545</t>
+          <t>16547</t>
         </is>
       </c>
       <c r="C833" s="7" t="inlineStr">
         <is>
-          <t>11174808</t>
+          <t>11177274</t>
         </is>
       </c>
       <c r="D833" t="inlineStr">
         <is>
-          <t>Wt26SSCC24Grad</t>
+          <t>Wt26SSCC24Win</t>
         </is>
       </c>
       <c r="E833" t="inlineStr">
@@ -29551,17 +29551,17 @@
       </c>
       <c r="B834" s="7" t="inlineStr">
         <is>
-          <t>16546</t>
+          <t>16548</t>
         </is>
       </c>
       <c r="C834" s="7" t="inlineStr">
         <is>
-          <t>11174811</t>
+          <t>11174801</t>
         </is>
       </c>
       <c r="D834" t="inlineStr">
         <is>
-          <t>Wt26SS30Jac</t>
+          <t>Wt26SSBTL20SV</t>
         </is>
       </c>
       <c r="E834" t="inlineStr">
@@ -29586,17 +29586,17 @@
       </c>
       <c r="B835" s="7" t="inlineStr">
         <is>
-          <t>16547</t>
+          <t>16549</t>
         </is>
       </c>
       <c r="C835" s="7" t="inlineStr">
         <is>
-          <t>11177274</t>
+          <t>11174803</t>
         </is>
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>Wt26SSCC24Win</t>
+          <t>Wt262PkStanley</t>
         </is>
       </c>
       <c r="E835" t="inlineStr">
@@ -29621,17 +29621,17 @@
       </c>
       <c r="B836" s="7" t="inlineStr">
         <is>
-          <t>16548</t>
+          <t>16550</t>
         </is>
       </c>
       <c r="C836" s="7" t="inlineStr">
         <is>
-          <t>11174801</t>
+          <t>11174776</t>
         </is>
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>Wt26SSBTL20SV</t>
+          <t>Wt26Mug14Bow</t>
         </is>
       </c>
       <c r="E836" t="inlineStr">
@@ -29656,17 +29656,17 @@
       </c>
       <c r="B837" s="7" t="inlineStr">
         <is>
-          <t>16549</t>
+          <t>16551</t>
         </is>
       </c>
       <c r="C837" s="7" t="inlineStr">
         <is>
-          <t>11174803</t>
+          <t>11174775</t>
         </is>
       </c>
       <c r="D837" t="inlineStr">
         <is>
-          <t>Wt262PkStanley</t>
+          <t>Wt26Dw12Jac</t>
         </is>
       </c>
       <c r="E837" t="inlineStr">
@@ -29691,17 +29691,17 @@
       </c>
       <c r="B838" s="7" t="inlineStr">
         <is>
-          <t>16550</t>
+          <t>16552</t>
         </is>
       </c>
       <c r="C838" s="7" t="inlineStr">
         <is>
-          <t>11174776</t>
+          <t>11174798</t>
         </is>
       </c>
       <c r="D838" t="inlineStr">
         <is>
-          <t>Wt26Mug14Bow</t>
+          <t>Wt26SS16Green</t>
         </is>
       </c>
       <c r="E838" t="inlineStr">
@@ -29726,17 +29726,17 @@
       </c>
       <c r="B839" s="7" t="inlineStr">
         <is>
-          <t>16551</t>
+          <t>16553</t>
         </is>
       </c>
       <c r="C839" s="7" t="inlineStr">
         <is>
-          <t>11174775</t>
+          <t>11174800</t>
         </is>
       </c>
       <c r="D839" t="inlineStr">
         <is>
-          <t>Wt26Dw12Jac</t>
+          <t>Wt26BTL20Gr</t>
         </is>
       </c>
       <c r="E839" t="inlineStr">
@@ -29761,17 +29761,17 @@
       </c>
       <c r="B840" s="7" t="inlineStr">
         <is>
-          <t>16552</t>
+          <t>16554</t>
         </is>
       </c>
       <c r="C840" s="7" t="inlineStr">
         <is>
-          <t>11174798</t>
+          <t>11174807</t>
         </is>
       </c>
       <c r="D840" t="inlineStr">
         <is>
-          <t>Wt26SS16Green</t>
+          <t>Wt26SS16Choco</t>
         </is>
       </c>
       <c r="E840" t="inlineStr">
@@ -29796,17 +29796,17 @@
       </c>
       <c r="B841" s="7" t="inlineStr">
         <is>
-          <t>16553</t>
+          <t>16555</t>
         </is>
       </c>
       <c r="C841" s="7" t="inlineStr">
         <is>
-          <t>11174800</t>
+          <t>11174810</t>
         </is>
       </c>
       <c r="D841" t="inlineStr">
         <is>
-          <t>Wt26BTL20Gr</t>
+          <t>Wt26Canteen</t>
         </is>
       </c>
       <c r="E841" t="inlineStr">
@@ -29831,17 +29831,17 @@
       </c>
       <c r="B842" s="7" t="inlineStr">
         <is>
-          <t>16554</t>
+          <t>16556</t>
         </is>
       </c>
       <c r="C842" s="7" t="inlineStr">
         <is>
-          <t>11174807</t>
+          <t>11174799</t>
         </is>
       </c>
       <c r="D842" t="inlineStr">
         <is>
-          <t>Wt26SS16Choco</t>
+          <t>Wt26SSCC16Grad</t>
         </is>
       </c>
       <c r="E842" t="inlineStr">
@@ -29866,17 +29866,17 @@
       </c>
       <c r="B843" s="7" t="inlineStr">
         <is>
-          <t>16555</t>
+          <t>16557</t>
         </is>
       </c>
       <c r="C843" s="7" t="inlineStr">
         <is>
-          <t>11174810</t>
+          <t>11174806</t>
         </is>
       </c>
       <c r="D843" t="inlineStr">
         <is>
-          <t>Wt26Canteen</t>
+          <t>Wt26SSCC16Jac</t>
         </is>
       </c>
       <c r="E843" t="inlineStr">
@@ -29901,17 +29901,17 @@
       </c>
       <c r="B844" s="7" t="inlineStr">
         <is>
-          <t>16556</t>
+          <t>16558</t>
         </is>
       </c>
       <c r="C844" s="7" t="inlineStr">
         <is>
-          <t>11174799</t>
+          <t>11177275</t>
         </is>
       </c>
       <c r="D844" t="inlineStr">
         <is>
-          <t>Wt26SSCC16Grad</t>
+          <t>Wt26SS20SV</t>
         </is>
       </c>
       <c r="E844" t="inlineStr">
@@ -29936,17 +29936,17 @@
       </c>
       <c r="B845" s="7" t="inlineStr">
         <is>
-          <t>16557</t>
+          <t>16559</t>
         </is>
       </c>
       <c r="C845" s="7" t="inlineStr">
         <is>
-          <t>11174806</t>
+          <t>11177276</t>
         </is>
       </c>
       <c r="D845" t="inlineStr">
         <is>
-          <t>Wt26SSCC16Jac</t>
+          <t>Wt26SS20Jac</t>
         </is>
       </c>
       <c r="E845" t="inlineStr">
@@ -29971,17 +29971,17 @@
       </c>
       <c r="B846" s="7" t="inlineStr">
         <is>
-          <t>16558</t>
+          <t>16572</t>
         </is>
       </c>
       <c r="C846" s="7" t="inlineStr">
         <is>
-          <t>11177275</t>
+          <t>11174791</t>
         </is>
       </c>
       <c r="D846" t="inlineStr">
         <is>
-          <t>Wt26SS20SV</t>
+          <t>Wt26ReusSV</t>
         </is>
       </c>
       <c r="E846" t="inlineStr">
@@ -30006,17 +30006,17 @@
       </c>
       <c r="B847" s="7" t="inlineStr">
         <is>
-          <t>16559</t>
+          <t>16573</t>
         </is>
       </c>
       <c r="C847" s="7" t="inlineStr">
         <is>
-          <t>11177276</t>
+          <t>11175037</t>
         </is>
       </c>
       <c r="D847" t="inlineStr">
         <is>
-          <t>Wt26SS20Jac</t>
+          <t>Wt26Tu16Charm</t>
         </is>
       </c>
       <c r="E847" t="inlineStr">
@@ -30041,17 +30041,17 @@
       </c>
       <c r="B848" s="7" t="inlineStr">
         <is>
-          <t>16572</t>
+          <t>16588</t>
         </is>
       </c>
       <c r="C848" s="7" t="inlineStr">
         <is>
-          <t>11174791</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D848" t="inlineStr">
         <is>
-          <t>Wt26ReusSV</t>
+          <t>Xm25ReuElev</t>
         </is>
       </c>
       <c r="E848" t="inlineStr">
@@ -30076,17 +30076,17 @@
       </c>
       <c r="B849" s="7" t="inlineStr">
         <is>
-          <t>16573</t>
+          <t>16589</t>
         </is>
       </c>
       <c r="C849" s="7" t="inlineStr">
         <is>
-          <t>11175037</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D849" t="inlineStr">
         <is>
-          <t>Wt26Tu16Charm</t>
+          <t>Xm25ReuMike</t>
         </is>
       </c>
       <c r="E849" t="inlineStr">
@@ -30111,7 +30111,7 @@
       </c>
       <c r="B850" s="7" t="inlineStr">
         <is>
-          <t>16588</t>
+          <t>16590</t>
         </is>
       </c>
       <c r="C850" s="7" t="inlineStr">
@@ -30121,7 +30121,7 @@
       </c>
       <c r="D850" t="inlineStr">
         <is>
-          <t>Xm25ReuElev</t>
+          <t>Xm25Reus16ST</t>
         </is>
       </c>
       <c r="E850" t="inlineStr">
@@ -30146,7 +30146,7 @@
       </c>
       <c r="B851" s="7" t="inlineStr">
         <is>
-          <t>16589</t>
+          <t>16591</t>
         </is>
       </c>
       <c r="C851" s="7" t="inlineStr">
@@ -30156,7 +30156,7 @@
       </c>
       <c r="D851" t="inlineStr">
         <is>
-          <t>Xm25ReuMike</t>
+          <t>Xm25Reu24CCST</t>
         </is>
       </c>
       <c r="E851" t="inlineStr">
@@ -30181,7 +30181,7 @@
       </c>
       <c r="B852" s="7" t="inlineStr">
         <is>
-          <t>16590</t>
+          <t>16602</t>
         </is>
       </c>
       <c r="C852" s="7" t="inlineStr">
@@ -30191,7 +30191,7 @@
       </c>
       <c r="D852" t="inlineStr">
         <is>
-          <t>Xm25Reus16ST</t>
+          <t>Xm25Reu2Hol</t>
         </is>
       </c>
       <c r="E852" t="inlineStr">
@@ -30216,7 +30216,7 @@
       </c>
       <c r="B853" s="7" t="inlineStr">
         <is>
-          <t>16591</t>
+          <t>16603</t>
         </is>
       </c>
       <c r="C853" s="7" t="inlineStr">
@@ -30226,7 +30226,7 @@
       </c>
       <c r="D853" t="inlineStr">
         <is>
-          <t>Xm25Reu24CCST</t>
+          <t>Xm25Reu1Hol</t>
         </is>
       </c>
       <c r="E853" t="inlineStr">
@@ -30251,17 +30251,17 @@
       </c>
       <c r="B854" s="7" t="inlineStr">
         <is>
-          <t>16602</t>
+          <t>16607</t>
         </is>
       </c>
       <c r="C854" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11177964</t>
         </is>
       </c>
       <c r="D854" t="inlineStr">
         <is>
-          <t>Xm25Reu2Hol</t>
+          <t>Sp26WTBLSS16Cher</t>
         </is>
       </c>
       <c r="E854" t="inlineStr">
@@ -30286,17 +30286,17 @@
       </c>
       <c r="B855" s="7" t="inlineStr">
         <is>
-          <t>16603</t>
+          <t>16608</t>
         </is>
       </c>
       <c r="C855" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11176612</t>
         </is>
       </c>
       <c r="D855" t="inlineStr">
         <is>
-          <t>Xm25Reu1Hol</t>
+          <t>Wt26CC15Blue</t>
         </is>
       </c>
       <c r="E855" t="inlineStr">
@@ -30321,17 +30321,17 @@
       </c>
       <c r="B856" s="7" t="inlineStr">
         <is>
-          <t>16607</t>
+          <t>16609</t>
         </is>
       </c>
       <c r="C856" s="7" t="inlineStr">
         <is>
-          <t>11177964</t>
+          <t>11176610</t>
         </is>
       </c>
       <c r="D856" t="inlineStr">
         <is>
-          <t>Sp26WTBLSS16Cher</t>
+          <t>Wt26TuSS16Duck</t>
         </is>
       </c>
       <c r="E856" t="inlineStr">
@@ -30356,17 +30356,17 @@
       </c>
       <c r="B857" s="7" t="inlineStr">
         <is>
-          <t>16608</t>
+          <t>16610</t>
         </is>
       </c>
       <c r="C857" s="7" t="inlineStr">
         <is>
-          <t>11176612</t>
+          <t>11179880</t>
         </is>
       </c>
       <c r="D857" t="inlineStr">
         <is>
-          <t>Wt26CC15Blue</t>
+          <t>SII26SS16Resort</t>
         </is>
       </c>
       <c r="E857" t="inlineStr">
@@ -30391,17 +30391,17 @@
       </c>
       <c r="B858" s="7" t="inlineStr">
         <is>
-          <t>16609</t>
+          <t>16611</t>
         </is>
       </c>
       <c r="C858" s="7" t="inlineStr">
         <is>
-          <t>11176610</t>
+          <t>11177937</t>
         </is>
       </c>
       <c r="D858" t="inlineStr">
         <is>
-          <t>Wt26TuSS16Duck</t>
+          <t>Sp26CCup16Cherry</t>
         </is>
       </c>
       <c r="E858" t="inlineStr">
@@ -30426,17 +30426,17 @@
       </c>
       <c r="B859" s="7" t="inlineStr">
         <is>
-          <t>16610</t>
+          <t>16613</t>
         </is>
       </c>
       <c r="C859" s="7" t="inlineStr">
         <is>
-          <t>11179880</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D859" t="inlineStr">
         <is>
-          <t>SII26SS16Resort</t>
+          <t>Xm25StopDermo</t>
         </is>
       </c>
       <c r="E859" t="inlineStr">
@@ -30461,17 +30461,17 @@
       </c>
       <c r="B860" s="7" t="inlineStr">
         <is>
-          <t>16611</t>
+          <t>16614</t>
         </is>
       </c>
       <c r="C860" s="7" t="inlineStr">
         <is>
-          <t>11177937</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D860" t="inlineStr">
         <is>
-          <t>Sp26CCup16Cherry</t>
+          <t>Xm25StopHopp</t>
         </is>
       </c>
       <c r="E860" t="inlineStr">
@@ -30496,17 +30496,17 @@
       </c>
       <c r="B861" s="7" t="inlineStr">
         <is>
-          <t>16613</t>
+          <t>16658</t>
         </is>
       </c>
       <c r="C861" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11176708</t>
         </is>
       </c>
       <c r="D861" t="inlineStr">
         <is>
-          <t>Xm25StopDermo</t>
+          <t>Wt26GlassCC16</t>
         </is>
       </c>
       <c r="E861" t="inlineStr">
@@ -30531,17 +30531,17 @@
       </c>
       <c r="B862" s="7" t="inlineStr">
         <is>
-          <t>16614</t>
+          <t>16659</t>
         </is>
       </c>
       <c r="C862" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11176714</t>
         </is>
       </c>
       <c r="D862" t="inlineStr">
         <is>
-          <t>Xm25StopHopp</t>
+          <t>Wt26SS16Vac</t>
         </is>
       </c>
       <c r="E862" t="inlineStr">
@@ -30566,17 +30566,17 @@
       </c>
       <c r="B863" s="7" t="inlineStr">
         <is>
-          <t>16658</t>
+          <t>16660</t>
         </is>
       </c>
       <c r="C863" s="7" t="inlineStr">
         <is>
-          <t>11176708</t>
+          <t>11176719</t>
         </is>
       </c>
       <c r="D863" t="inlineStr">
         <is>
-          <t>Wt26GlassCC16</t>
+          <t>Wt26SSCC24CarryL</t>
         </is>
       </c>
       <c r="E863" t="inlineStr">
@@ -30601,17 +30601,17 @@
       </c>
       <c r="B864" s="7" t="inlineStr">
         <is>
-          <t>16659</t>
+          <t>16661</t>
         </is>
       </c>
       <c r="C864" s="7" t="inlineStr">
         <is>
-          <t>11176714</t>
+          <t>11176720</t>
         </is>
       </c>
       <c r="D864" t="inlineStr">
         <is>
-          <t>Wt26SS16Vac</t>
+          <t>Wt26SSCC30Togo</t>
         </is>
       </c>
       <c r="E864" t="inlineStr">
@@ -30636,17 +30636,17 @@
       </c>
       <c r="B865" s="7" t="inlineStr">
         <is>
-          <t>16660</t>
+          <t>16662</t>
         </is>
       </c>
       <c r="C865" s="7" t="inlineStr">
         <is>
-          <t>11176719</t>
+          <t>11176721</t>
         </is>
       </c>
       <c r="D865" t="inlineStr">
         <is>
-          <t>Wt26SSCC24CarryL</t>
+          <t>Sp26Stan30Purp</t>
         </is>
       </c>
       <c r="E865" t="inlineStr">
@@ -30671,17 +30671,17 @@
       </c>
       <c r="B866" s="7" t="inlineStr">
         <is>
-          <t>16661</t>
+          <t>16663</t>
         </is>
       </c>
       <c r="C866" s="7" t="inlineStr">
         <is>
-          <t>11176720</t>
+          <t>11176699</t>
         </is>
       </c>
       <c r="D866" t="inlineStr">
         <is>
-          <t>Wt26SSCC30Togo</t>
+          <t>Sp26Mug14Rabbit</t>
         </is>
       </c>
       <c r="E866" t="inlineStr">
@@ -30706,17 +30706,17 @@
       </c>
       <c r="B867" s="7" t="inlineStr">
         <is>
-          <t>16662</t>
+          <t>16665</t>
         </is>
       </c>
       <c r="C867" s="7" t="inlineStr">
         <is>
-          <t>11176721</t>
+          <t>11176701</t>
         </is>
       </c>
       <c r="D867" t="inlineStr">
         <is>
-          <t>Sp26Stan30Purp</t>
+          <t>Sp26CC216Rabbit</t>
         </is>
       </c>
       <c r="E867" t="inlineStr">
@@ -30741,17 +30741,17 @@
       </c>
       <c r="B868" s="7" t="inlineStr">
         <is>
-          <t>16663</t>
+          <t>16666</t>
         </is>
       </c>
       <c r="C868" s="7" t="inlineStr">
         <is>
-          <t>11176699</t>
+          <t>11176702</t>
         </is>
       </c>
       <c r="D868" t="inlineStr">
         <is>
-          <t>Sp26Mug14Rabbit</t>
+          <t>Sp26Tu20Blue</t>
         </is>
       </c>
       <c r="E868" t="inlineStr">
@@ -30776,17 +30776,17 @@
       </c>
       <c r="B869" s="7" t="inlineStr">
         <is>
-          <t>16664</t>
+          <t>16667</t>
         </is>
       </c>
       <c r="C869" s="7" t="inlineStr">
         <is>
-          <t>11176710</t>
+          <t>11176715</t>
         </is>
       </c>
       <c r="D869" t="inlineStr">
         <is>
-          <t>Sp26CC24Dome</t>
+          <t>Sp26SS16Rabbit</t>
         </is>
       </c>
       <c r="E869" t="inlineStr">
@@ -30811,17 +30811,17 @@
       </c>
       <c r="B870" s="7" t="inlineStr">
         <is>
-          <t>16665</t>
+          <t>16669</t>
         </is>
       </c>
       <c r="C870" s="7" t="inlineStr">
         <is>
-          <t>11176701</t>
+          <t>11176711</t>
         </is>
       </c>
       <c r="D870" t="inlineStr">
         <is>
-          <t>Sp26CC216Rabbit</t>
+          <t>Sp26Gl18Mottled</t>
         </is>
       </c>
       <c r="E870" t="inlineStr">
@@ -30846,17 +30846,17 @@
       </c>
       <c r="B871" s="7" t="inlineStr">
         <is>
-          <t>16666</t>
+          <t>16670</t>
         </is>
       </c>
       <c r="C871" s="7" t="inlineStr">
         <is>
-          <t>11176702</t>
+          <t>11176700</t>
         </is>
       </c>
       <c r="D871" t="inlineStr">
         <is>
-          <t>Sp26Tu20Blue</t>
+          <t>Sp26Tz14GlassC</t>
         </is>
       </c>
       <c r="E871" t="inlineStr">
@@ -30881,17 +30881,17 @@
       </c>
       <c r="B872" s="7" t="inlineStr">
         <is>
-          <t>16667</t>
+          <t>16671</t>
         </is>
       </c>
       <c r="C872" s="7" t="inlineStr">
         <is>
-          <t>11176715</t>
+          <t>11176717</t>
         </is>
       </c>
       <c r="D872" t="inlineStr">
         <is>
-          <t>Sp26SS16Rabbit</t>
+          <t>Sp26SS12Pink</t>
         </is>
       </c>
       <c r="E872" t="inlineStr">
@@ -30916,17 +30916,17 @@
       </c>
       <c r="B873" s="7" t="inlineStr">
         <is>
-          <t>16669</t>
+          <t>16672</t>
         </is>
       </c>
       <c r="C873" s="7" t="inlineStr">
         <is>
-          <t>11176711</t>
+          <t>11176724</t>
         </is>
       </c>
       <c r="D873" t="inlineStr">
         <is>
-          <t>Sp26Gl18Mottled</t>
+          <t>Sp26CookieJP</t>
         </is>
       </c>
       <c r="E873" t="inlineStr">
@@ -30951,17 +30951,17 @@
       </c>
       <c r="B874" s="7" t="inlineStr">
         <is>
-          <t>16670</t>
+          <t>16673</t>
         </is>
       </c>
       <c r="C874" s="7" t="inlineStr">
         <is>
-          <t>11176700</t>
+          <t>11176703</t>
         </is>
       </c>
       <c r="D874" t="inlineStr">
         <is>
-          <t>Sp26Tz14GlassC</t>
+          <t>Sp26Tu16Cherry</t>
         </is>
       </c>
       <c r="E874" t="inlineStr">
@@ -30986,17 +30986,17 @@
       </c>
       <c r="B875" s="7" t="inlineStr">
         <is>
-          <t>16671</t>
+          <t>16674</t>
         </is>
       </c>
       <c r="C875" s="7" t="inlineStr">
         <is>
-          <t>11176717</t>
+          <t>11176704</t>
         </is>
       </c>
       <c r="D875" t="inlineStr">
         <is>
-          <t>Sp26SS12Pink</t>
+          <t>Sp26CC16Prism</t>
         </is>
       </c>
       <c r="E875" t="inlineStr">
@@ -31021,17 +31021,17 @@
       </c>
       <c r="B876" s="7" t="inlineStr">
         <is>
-          <t>16672</t>
+          <t>16675</t>
         </is>
       </c>
       <c r="C876" s="7" t="inlineStr">
         <is>
-          <t>11176724</t>
+          <t>11176722</t>
         </is>
       </c>
       <c r="D876" t="inlineStr">
         <is>
-          <t>Sp26CookieJP</t>
+          <t>Sp26SSCC24Cherry</t>
         </is>
       </c>
       <c r="E876" t="inlineStr">
@@ -31056,17 +31056,17 @@
       </c>
       <c r="B877" s="7" t="inlineStr">
         <is>
-          <t>16673</t>
+          <t>16676</t>
         </is>
       </c>
       <c r="C877" s="7" t="inlineStr">
         <is>
-          <t>11176703</t>
+          <t>11176718</t>
         </is>
       </c>
       <c r="D877" t="inlineStr">
         <is>
-          <t>Sp26Tu16Cherry</t>
+          <t>Sp26SS16Cherry</t>
         </is>
       </c>
       <c r="E877" t="inlineStr">
@@ -31091,17 +31091,17 @@
       </c>
       <c r="B878" s="7" t="inlineStr">
         <is>
-          <t>16674</t>
+          <t>16677</t>
         </is>
       </c>
       <c r="C878" s="7" t="inlineStr">
         <is>
-          <t>11176704</t>
+          <t>11176723</t>
         </is>
       </c>
       <c r="D878" t="inlineStr">
         <is>
-          <t>Sp26CC16Prism</t>
+          <t>Sp26SSVac40Cherr</t>
         </is>
       </c>
       <c r="E878" t="inlineStr">
@@ -31126,17 +31126,17 @@
       </c>
       <c r="B879" s="7" t="inlineStr">
         <is>
-          <t>16675</t>
+          <t>16678</t>
         </is>
       </c>
       <c r="C879" s="7" t="inlineStr">
         <is>
-          <t>11176722</t>
+          <t>11176705</t>
         </is>
       </c>
       <c r="D879" t="inlineStr">
         <is>
-          <t>Sp26SSCC24Cherry</t>
+          <t>Sp26ReusTierra</t>
         </is>
       </c>
       <c r="E879" t="inlineStr">
@@ -31161,17 +31161,17 @@
       </c>
       <c r="B880" s="7" t="inlineStr">
         <is>
-          <t>16676</t>
+          <t>16679</t>
         </is>
       </c>
       <c r="C880" s="7" t="inlineStr">
         <is>
-          <t>11176718</t>
+          <t>11176712</t>
         </is>
       </c>
       <c r="D880" t="inlineStr">
         <is>
-          <t>Sp26SS16Cherry</t>
+          <t>Sp26CCReusTierra</t>
         </is>
       </c>
       <c r="E880" t="inlineStr">
@@ -31196,17 +31196,17 @@
       </c>
       <c r="B881" s="7" t="inlineStr">
         <is>
-          <t>16677</t>
+          <t>16680</t>
         </is>
       </c>
       <c r="C881" s="7" t="inlineStr">
         <is>
-          <t>11176723</t>
+          <t>11177607</t>
         </is>
       </c>
       <c r="D881" t="inlineStr">
         <is>
-          <t>Sp26SSVac40Cherr</t>
+          <t>Wt26ReusSiren</t>
         </is>
       </c>
       <c r="E881" t="inlineStr">
@@ -31231,17 +31231,17 @@
       </c>
       <c r="B882" s="7" t="inlineStr">
         <is>
-          <t>16678</t>
+          <t>16719</t>
         </is>
       </c>
       <c r="C882" s="7" t="inlineStr">
         <is>
-          <t>11176705</t>
+          <t>11176586</t>
         </is>
       </c>
       <c r="D882" t="inlineStr">
         <is>
-          <t>Sp26ReusTierra</t>
+          <t>SII26SSCC20Pony</t>
         </is>
       </c>
       <c r="E882" t="inlineStr">
@@ -31266,17 +31266,17 @@
       </c>
       <c r="B883" s="7" t="inlineStr">
         <is>
-          <t>16679</t>
+          <t>16720</t>
         </is>
       </c>
       <c r="C883" s="7" t="inlineStr">
         <is>
-          <t>11176712</t>
+          <t>11176587</t>
         </is>
       </c>
       <c r="D883" t="inlineStr">
         <is>
-          <t>Sp26CCReusTierra</t>
+          <t>SII26SSCC16Pony</t>
         </is>
       </c>
       <c r="E883" t="inlineStr">
@@ -31301,17 +31301,17 @@
       </c>
       <c r="B884" s="7" t="inlineStr">
         <is>
-          <t>16680</t>
+          <t>16721</t>
         </is>
       </c>
       <c r="C884" s="7" t="inlineStr">
         <is>
-          <t>11177607</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D884" t="inlineStr">
         <is>
-          <t>Wt26ReusSiren</t>
+          <t>Sp26SS16Under</t>
         </is>
       </c>
       <c r="E884" t="inlineStr">
@@ -31336,17 +31336,17 @@
       </c>
       <c r="B885" s="7" t="inlineStr">
         <is>
-          <t>16719</t>
+          <t>16729</t>
         </is>
       </c>
       <c r="C885" s="7" t="inlineStr">
         <is>
-          <t>11176586</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D885" t="inlineStr">
         <is>
-          <t>SII26SSCC20Pony</t>
+          <t>Wt26ReusBear</t>
         </is>
       </c>
       <c r="E885" t="inlineStr">
@@ -31371,17 +31371,17 @@
       </c>
       <c r="B886" s="7" t="inlineStr">
         <is>
-          <t>16720</t>
+          <t>16769</t>
         </is>
       </c>
       <c r="C886" s="7" t="inlineStr">
         <is>
-          <t>11176587</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D886" t="inlineStr">
         <is>
-          <t>SII26SSCC16Pony</t>
+          <t>Wt26VasoPistache</t>
         </is>
       </c>
       <c r="E886" t="inlineStr">
@@ -31406,7 +31406,7 @@
       </c>
       <c r="B887" s="7" t="inlineStr">
         <is>
-          <t>16721</t>
+          <t>16770</t>
         </is>
       </c>
       <c r="C887" s="7" t="inlineStr">
@@ -31416,7 +31416,7 @@
       </c>
       <c r="D887" t="inlineStr">
         <is>
-          <t>Sp26SS16Under</t>
+          <t>Wt26VasoFresa</t>
         </is>
       </c>
       <c r="E887" t="inlineStr">
@@ -31441,7 +31441,7 @@
       </c>
       <c r="B888" s="7" t="inlineStr">
         <is>
-          <t>16729</t>
+          <t>16771</t>
         </is>
       </c>
       <c r="C888" s="7" t="inlineStr">
@@ -31451,7 +31451,7 @@
       </c>
       <c r="D888" t="inlineStr">
         <is>
-          <t>Wt26ReusBear</t>
+          <t>Wt26VasoJacaran</t>
         </is>
       </c>
       <c r="E888" t="inlineStr">
@@ -31476,7 +31476,7 @@
       </c>
       <c r="B889" s="7" t="inlineStr">
         <is>
-          <t>16769</t>
+          <t>16775</t>
         </is>
       </c>
       <c r="C889" s="7" t="inlineStr">
@@ -31486,7 +31486,7 @@
       </c>
       <c r="D889" t="inlineStr">
         <is>
-          <t>Wt26VasoPistache</t>
+          <t>Wt26LlaveroSV</t>
         </is>
       </c>
       <c r="E889" t="inlineStr">
@@ -31511,17 +31511,17 @@
       </c>
       <c r="B890" s="7" t="inlineStr">
         <is>
-          <t>16770</t>
+          <t>16777</t>
         </is>
       </c>
       <c r="C890" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11179885</t>
         </is>
       </c>
       <c r="D890" t="inlineStr">
         <is>
-          <t>Wt26VasoFresa</t>
+          <t>SII26BTL20Resort</t>
         </is>
       </c>
       <c r="E890" t="inlineStr">
@@ -31546,17 +31546,17 @@
       </c>
       <c r="B891" s="7" t="inlineStr">
         <is>
-          <t>16771</t>
+          <t>16779</t>
         </is>
       </c>
       <c r="C891" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11176592</t>
         </is>
       </c>
       <c r="D891" t="inlineStr">
         <is>
-          <t>Wt26VasoJacaran</t>
+          <t>SII26SSTu12Pony</t>
         </is>
       </c>
       <c r="E891" t="inlineStr">
@@ -31581,7 +31581,7 @@
       </c>
       <c r="B892" s="7" t="inlineStr">
         <is>
-          <t>16775</t>
+          <t>16780</t>
         </is>
       </c>
       <c r="C892" s="7" t="inlineStr">
@@ -31591,7 +31591,7 @@
       </c>
       <c r="D892" t="inlineStr">
         <is>
-          <t>Wt26LlaveroSV</t>
+          <t>Sp26WTBL19Under</t>
         </is>
       </c>
       <c r="E892" t="inlineStr">
@@ -31616,17 +31616,17 @@
       </c>
       <c r="B893" s="7" t="inlineStr">
         <is>
-          <t>16777</t>
+          <t>16781</t>
         </is>
       </c>
       <c r="C893" s="7" t="inlineStr">
         <is>
-          <t>11179885</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D893" t="inlineStr">
         <is>
-          <t>SII26BTL20Resort</t>
+          <t>Sp26Tu20Blossom</t>
         </is>
       </c>
       <c r="E893" t="inlineStr">
@@ -31651,17 +31651,17 @@
       </c>
       <c r="B894" s="7" t="inlineStr">
         <is>
-          <t>16779</t>
+          <t>16784</t>
         </is>
       </c>
       <c r="C894" s="7" t="inlineStr">
         <is>
-          <t>11176592</t>
+          <t>11176597</t>
         </is>
       </c>
       <c r="D894" t="inlineStr">
         <is>
-          <t>SII26SSTu12Pony</t>
+          <t>SII26BearPony</t>
         </is>
       </c>
       <c r="E894" t="inlineStr">
@@ -31686,17 +31686,17 @@
       </c>
       <c r="B895" s="7" t="inlineStr">
         <is>
-          <t>16780</t>
+          <t>16793</t>
         </is>
       </c>
       <c r="C895" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>1176593</t>
         </is>
       </c>
       <c r="D895" t="inlineStr">
         <is>
-          <t>Sp26WTBL19Under</t>
+          <t>SII26BTL16Pony</t>
         </is>
       </c>
       <c r="E895" t="inlineStr">
@@ -31721,17 +31721,17 @@
       </c>
       <c r="B896" s="7" t="inlineStr">
         <is>
-          <t>16781</t>
+          <t>16875</t>
         </is>
       </c>
       <c r="C896" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11178952</t>
         </is>
       </c>
       <c r="D896" t="inlineStr">
         <is>
-          <t>Sp26Tu20Blossom</t>
+          <t>WC26SSCC24Grad</t>
         </is>
       </c>
       <c r="E896" t="inlineStr">
@@ -31756,17 +31756,17 @@
       </c>
       <c r="B897" s="7" t="inlineStr">
         <is>
-          <t>16784</t>
+          <t>16876</t>
         </is>
       </c>
       <c r="C897" s="7" t="inlineStr">
         <is>
-          <t>11176597</t>
+          <t>11178953</t>
         </is>
       </c>
       <c r="D897" t="inlineStr">
         <is>
-          <t>SII26BearPony</t>
+          <t>Sp26SSCC24Oran</t>
         </is>
       </c>
       <c r="E897" t="inlineStr">
@@ -31791,17 +31791,17 @@
       </c>
       <c r="B898" s="7" t="inlineStr">
         <is>
-          <t>16793</t>
+          <t>16877</t>
         </is>
       </c>
       <c r="C898" s="7" t="inlineStr">
         <is>
-          <t>1176593</t>
+          <t>11178954</t>
         </is>
       </c>
       <c r="D898" t="inlineStr">
         <is>
-          <t>SII26BTL16Pony</t>
+          <t>Sp26SSCC24CarryC</t>
         </is>
       </c>
       <c r="E898" t="inlineStr">
@@ -31826,17 +31826,17 @@
       </c>
       <c r="B899" s="7" t="inlineStr">
         <is>
-          <t>16875</t>
+          <t>16878</t>
         </is>
       </c>
       <c r="C899" s="7" t="inlineStr">
         <is>
-          <t>11178952</t>
+          <t>11178921</t>
         </is>
       </c>
       <c r="D899" t="inlineStr">
         <is>
-          <t>WC26SSCC24Grad</t>
+          <t>Sp26Tu16Orange</t>
         </is>
       </c>
       <c r="E899" t="inlineStr">
@@ -31861,17 +31861,17 @@
       </c>
       <c r="B900" s="7" t="inlineStr">
         <is>
-          <t>16876</t>
+          <t>16879</t>
         </is>
       </c>
       <c r="C900" s="7" t="inlineStr">
         <is>
-          <t>11178953</t>
+          <t>11178922</t>
         </is>
       </c>
       <c r="D900" t="inlineStr">
         <is>
-          <t>Sp26SSCC24Oran</t>
+          <t>WC26Tu16Flower</t>
         </is>
       </c>
       <c r="E900" t="inlineStr">
@@ -31896,17 +31896,17 @@
       </c>
       <c r="B901" s="7" t="inlineStr">
         <is>
-          <t>16877</t>
+          <t>16880</t>
         </is>
       </c>
       <c r="C901" s="7" t="inlineStr">
         <is>
-          <t>11178954</t>
+          <t>11178928</t>
         </is>
       </c>
       <c r="D901" t="inlineStr">
         <is>
-          <t>Sp26SSCC24CarryC</t>
+          <t>WC26CC24Road</t>
         </is>
       </c>
       <c r="E901" t="inlineStr">
@@ -31931,17 +31931,17 @@
       </c>
       <c r="B902" s="7" t="inlineStr">
         <is>
-          <t>16878</t>
+          <t>16882</t>
         </is>
       </c>
       <c r="C902" s="7" t="inlineStr">
         <is>
-          <t>11178921</t>
+          <t>11178930</t>
         </is>
       </c>
       <c r="D902" t="inlineStr">
         <is>
-          <t>Sp26Tu16Orange</t>
+          <t>WC26CC24Pride</t>
         </is>
       </c>
       <c r="E902" t="inlineStr">
@@ -31966,17 +31966,17 @@
       </c>
       <c r="B903" s="7" t="inlineStr">
         <is>
-          <t>16879</t>
+          <t>16883</t>
         </is>
       </c>
       <c r="C903" s="7" t="inlineStr">
         <is>
-          <t>11178922</t>
+          <t>11178964</t>
         </is>
       </c>
       <c r="D903" t="inlineStr">
         <is>
-          <t>WC26Tu16Flower</t>
+          <t>Sp26KeychainOr</t>
         </is>
       </c>
       <c r="E903" t="inlineStr">
@@ -32001,17 +32001,17 @@
       </c>
       <c r="B904" s="7" t="inlineStr">
         <is>
-          <t>16880</t>
+          <t>16884</t>
         </is>
       </c>
       <c r="C904" s="7" t="inlineStr">
         <is>
-          <t>11178928</t>
+          <t>11178934</t>
         </is>
       </c>
       <c r="D904" t="inlineStr">
         <is>
-          <t>WC26CC24Road</t>
+          <t>SII26CC24GID</t>
         </is>
       </c>
       <c r="E904" t="inlineStr">
@@ -32036,17 +32036,17 @@
       </c>
       <c r="B905" s="7" t="inlineStr">
         <is>
-          <t>16882</t>
+          <t>16885</t>
         </is>
       </c>
       <c r="C905" s="7" t="inlineStr">
         <is>
-          <t>11178930</t>
+          <t>11179003</t>
         </is>
       </c>
       <c r="D905" t="inlineStr">
         <is>
-          <t>WC26CC24Pride</t>
+          <t>Sp26CC24Teach</t>
         </is>
       </c>
       <c r="E905" t="inlineStr">
@@ -32071,17 +32071,17 @@
       </c>
       <c r="B906" s="7" t="inlineStr">
         <is>
-          <t>16883</t>
+          <t>16896</t>
         </is>
       </c>
       <c r="C906" s="7" t="inlineStr">
         <is>
-          <t>11178964</t>
+          <t>11178970</t>
         </is>
       </c>
       <c r="D906" t="inlineStr">
         <is>
-          <t>Sp26KeychainOr</t>
+          <t>Sp26SSCC16Band</t>
         </is>
       </c>
       <c r="E906" t="inlineStr">
@@ -32106,17 +32106,17 @@
       </c>
       <c r="B907" s="7" t="inlineStr">
         <is>
-          <t>16884</t>
+          <t>16897</t>
         </is>
       </c>
       <c r="C907" s="7" t="inlineStr">
         <is>
-          <t>11178934</t>
+          <t>11178959</t>
         </is>
       </c>
       <c r="D907" t="inlineStr">
         <is>
-          <t>SII26CC24GID</t>
+          <t>WC26CCSS24Puffy</t>
         </is>
       </c>
       <c r="E907" t="inlineStr">
@@ -32141,17 +32141,17 @@
       </c>
       <c r="B908" s="7" t="inlineStr">
         <is>
-          <t>16885</t>
+          <t>16898</t>
         </is>
       </c>
       <c r="C908" s="7" t="inlineStr">
         <is>
-          <t>11179003</t>
+          <t>11178938</t>
         </is>
       </c>
       <c r="D908" t="inlineStr">
         <is>
-          <t>Sp26CC24Teach</t>
+          <t>Sp26Tu16Mom</t>
         </is>
       </c>
       <c r="E908" t="inlineStr">
@@ -32176,17 +32176,17 @@
       </c>
       <c r="B909" s="7" t="inlineStr">
         <is>
-          <t>16896</t>
+          <t>16899</t>
         </is>
       </c>
       <c r="C909" s="7" t="inlineStr">
         <is>
-          <t>11178970</t>
+          <t>11179004</t>
         </is>
       </c>
       <c r="D909" t="inlineStr">
         <is>
-          <t>Sp26SSCC16Band</t>
+          <t>Sp26Tu16Teach</t>
         </is>
       </c>
       <c r="E909" t="inlineStr">
@@ -32211,17 +32211,17 @@
       </c>
       <c r="B910" s="7" t="inlineStr">
         <is>
-          <t>16897</t>
+          <t>16900</t>
         </is>
       </c>
       <c r="C910" s="7" t="inlineStr">
         <is>
-          <t>11178959</t>
+          <t>11178941</t>
         </is>
       </c>
       <c r="D910" t="inlineStr">
         <is>
-          <t>WC26CCSS24Puffy</t>
+          <t>SII26SS16Studded</t>
         </is>
       </c>
       <c r="E910" t="inlineStr">
@@ -32246,17 +32246,17 @@
       </c>
       <c r="B911" s="7" t="inlineStr">
         <is>
-          <t>16898</t>
+          <t>16901</t>
         </is>
       </c>
       <c r="C911" s="7" t="inlineStr">
         <is>
-          <t>11178938</t>
+          <t>11178937</t>
         </is>
       </c>
       <c r="D911" t="inlineStr">
         <is>
-          <t>Sp26Tu16Mom</t>
+          <t>WC26Mug12Stan</t>
         </is>
       </c>
       <c r="E911" t="inlineStr">
@@ -32281,17 +32281,17 @@
       </c>
       <c r="B912" s="7" t="inlineStr">
         <is>
-          <t>16899</t>
+          <t>16902</t>
         </is>
       </c>
       <c r="C912" s="7" t="inlineStr">
         <is>
-          <t>11179004</t>
+          <t>11178920</t>
         </is>
       </c>
       <c r="D912" t="inlineStr">
         <is>
-          <t>Sp26Tu16Teach</t>
+          <t>WC26Tu20Yellow</t>
         </is>
       </c>
       <c r="E912" t="inlineStr">
@@ -32316,17 +32316,17 @@
       </c>
       <c r="B913" s="7" t="inlineStr">
         <is>
-          <t>16900</t>
+          <t>16903</t>
         </is>
       </c>
       <c r="C913" s="7" t="inlineStr">
         <is>
-          <t>11178941</t>
+          <t>11178926</t>
         </is>
       </c>
       <c r="D913" t="inlineStr">
         <is>
-          <t>SII26SS16Studded</t>
+          <t>Sp26CC24Or</t>
         </is>
       </c>
       <c r="E913" t="inlineStr">
@@ -32351,17 +32351,17 @@
       </c>
       <c r="B914" s="7" t="inlineStr">
         <is>
-          <t>16901</t>
+          <t>16904</t>
         </is>
       </c>
       <c r="C914" s="7" t="inlineStr">
         <is>
-          <t>11178937</t>
+          <t>11178965</t>
         </is>
       </c>
       <c r="D914" t="inlineStr">
         <is>
-          <t>WC26Mug12Stan</t>
+          <t>WC26ToteRoad</t>
         </is>
       </c>
       <c r="E914" t="inlineStr">
@@ -32386,17 +32386,17 @@
       </c>
       <c r="B915" s="7" t="inlineStr">
         <is>
-          <t>16902</t>
+          <t>16905</t>
         </is>
       </c>
       <c r="C915" s="7" t="inlineStr">
         <is>
-          <t>11178920</t>
+          <t>11178966</t>
         </is>
       </c>
       <c r="D915" t="inlineStr">
         <is>
-          <t>WC26Tu20Yellow</t>
+          <t>WC26TotePride</t>
         </is>
       </c>
       <c r="E915" t="inlineStr">
@@ -32421,17 +32421,17 @@
       </c>
       <c r="B916" s="7" t="inlineStr">
         <is>
-          <t>16903</t>
+          <t>16906</t>
         </is>
       </c>
       <c r="C916" s="7" t="inlineStr">
         <is>
-          <t>11178926</t>
+          <t>11179005</t>
         </is>
       </c>
       <c r="D916" t="inlineStr">
         <is>
-          <t>Sp26CC24Or</t>
+          <t>WC26SS30Pride</t>
         </is>
       </c>
       <c r="E916" t="inlineStr">
@@ -32456,17 +32456,17 @@
       </c>
       <c r="B917" s="7" t="inlineStr">
         <is>
-          <t>16904</t>
+          <t>16908</t>
         </is>
       </c>
       <c r="C917" s="7" t="inlineStr">
         <is>
-          <t>11178965</t>
+          <t>11187369</t>
         </is>
       </c>
       <c r="D917" t="inlineStr">
         <is>
-          <t>WC26ToteRoad</t>
+          <t>WC26BearWC</t>
         </is>
       </c>
       <c r="E917" t="inlineStr">
@@ -32491,17 +32491,17 @@
       </c>
       <c r="B918" s="7" t="inlineStr">
         <is>
-          <t>16905</t>
+          <t>16909</t>
         </is>
       </c>
       <c r="C918" s="7" t="inlineStr">
         <is>
-          <t>11178966</t>
+          <t>11178944</t>
         </is>
       </c>
       <c r="D918" t="inlineStr">
         <is>
-          <t>WC26TotePride</t>
+          <t>WC26SS20BTL</t>
         </is>
       </c>
       <c r="E918" t="inlineStr">
@@ -32526,17 +32526,17 @@
       </c>
       <c r="B919" s="7" t="inlineStr">
         <is>
-          <t>16906</t>
+          <t>16910</t>
         </is>
       </c>
       <c r="C919" s="7" t="inlineStr">
         <is>
-          <t>11179005</t>
+          <t>11178969</t>
         </is>
       </c>
       <c r="D919" t="inlineStr">
         <is>
-          <t>WC26SS30Pride</t>
+          <t>WC26SS16Pink</t>
         </is>
       </c>
       <c r="E919" t="inlineStr">
@@ -32561,17 +32561,17 @@
       </c>
       <c r="B920" s="7" t="inlineStr">
         <is>
-          <t>16908</t>
+          <t>16911</t>
         </is>
       </c>
       <c r="C920" s="7" t="inlineStr">
         <is>
-          <t>11187369</t>
+          <t>11178971</t>
         </is>
       </c>
       <c r="D920" t="inlineStr">
         <is>
-          <t>WC26BearWC</t>
+          <t>WC26SS16Charm</t>
         </is>
       </c>
       <c r="E920" t="inlineStr">
@@ -32596,17 +32596,17 @@
       </c>
       <c r="B921" s="7" t="inlineStr">
         <is>
-          <t>16909</t>
+          <t>16912</t>
         </is>
       </c>
       <c r="C921" s="7" t="inlineStr">
         <is>
-          <t>11178944</t>
+          <t>11178949</t>
         </is>
       </c>
       <c r="D921" t="inlineStr">
         <is>
-          <t>WC26SS20BTL</t>
+          <t>WC26SS20Pull</t>
         </is>
       </c>
       <c r="E921" t="inlineStr">
@@ -32631,17 +32631,17 @@
       </c>
       <c r="B922" s="7" t="inlineStr">
         <is>
-          <t>16910</t>
+          <t>16913</t>
         </is>
       </c>
       <c r="C922" s="7" t="inlineStr">
         <is>
-          <t>11178969</t>
+          <t>11178946</t>
         </is>
       </c>
       <c r="D922" t="inlineStr">
         <is>
-          <t>WC26SS16Pink</t>
+          <t>WC26SS20Twist</t>
         </is>
       </c>
       <c r="E922" t="inlineStr">
@@ -32666,17 +32666,17 @@
       </c>
       <c r="B923" s="7" t="inlineStr">
         <is>
-          <t>16911</t>
+          <t>16914</t>
         </is>
       </c>
       <c r="C923" s="7" t="inlineStr">
         <is>
-          <t>11178971</t>
+          <t>11178947</t>
         </is>
       </c>
       <c r="D923" t="inlineStr">
         <is>
-          <t>WC26SS16Charm</t>
+          <t>Sp26StanQuen20</t>
         </is>
       </c>
       <c r="E923" t="inlineStr">
@@ -32701,17 +32701,17 @@
       </c>
       <c r="B924" s="7" t="inlineStr">
         <is>
-          <t>16912</t>
+          <t>16915</t>
         </is>
       </c>
       <c r="C924" s="7" t="inlineStr">
         <is>
-          <t>11178949</t>
+          <t>11178948</t>
         </is>
       </c>
       <c r="D924" t="inlineStr">
         <is>
-          <t>WC26SS20Pull</t>
+          <t>WC26StanHand20</t>
         </is>
       </c>
       <c r="E924" t="inlineStr">
@@ -32736,17 +32736,17 @@
       </c>
       <c r="B925" s="7" t="inlineStr">
         <is>
-          <t>16913</t>
+          <t>16916</t>
         </is>
       </c>
       <c r="C925" s="7" t="inlineStr">
         <is>
-          <t>11178946</t>
+          <t>11178956</t>
         </is>
       </c>
       <c r="D925" t="inlineStr">
         <is>
-          <t>WC26SS20Twist</t>
+          <t>SII26Quencher30P</t>
         </is>
       </c>
       <c r="E925" t="inlineStr">
@@ -32771,17 +32771,17 @@
       </c>
       <c r="B926" s="7" t="inlineStr">
         <is>
-          <t>16914</t>
+          <t>16917</t>
         </is>
       </c>
       <c r="C926" s="7" t="inlineStr">
         <is>
-          <t>11178947</t>
+          <t>11178972</t>
         </is>
       </c>
       <c r="D926" t="inlineStr">
         <is>
-          <t>Sp26StanQuen20</t>
+          <t>Sp26Vac16Stan</t>
         </is>
       </c>
       <c r="E926" t="inlineStr">
@@ -32806,17 +32806,17 @@
       </c>
       <c r="B927" s="7" t="inlineStr">
         <is>
-          <t>16915</t>
+          <t>16918</t>
         </is>
       </c>
       <c r="C927" s="7" t="inlineStr">
         <is>
-          <t>11178948</t>
+          <t>11178943</t>
         </is>
       </c>
       <c r="D927" t="inlineStr">
         <is>
-          <t>WC26StanHand20</t>
+          <t>Sp26SS20Orange</t>
         </is>
       </c>
       <c r="E927" t="inlineStr">
@@ -32841,17 +32841,17 @@
       </c>
       <c r="B928" s="7" t="inlineStr">
         <is>
-          <t>16916</t>
+          <t>16919</t>
         </is>
       </c>
       <c r="C928" s="7" t="inlineStr">
         <is>
-          <t>11178956</t>
+          <t>11178957</t>
         </is>
       </c>
       <c r="D928" t="inlineStr">
         <is>
-          <t>SII26Quencher30P</t>
+          <t>WC26StanQuen30</t>
         </is>
       </c>
       <c r="E928" t="inlineStr">
@@ -32876,17 +32876,17 @@
       </c>
       <c r="B929" s="7" t="inlineStr">
         <is>
-          <t>16917</t>
+          <t>16920</t>
         </is>
       </c>
       <c r="C929" s="7" t="inlineStr">
         <is>
-          <t>11178972</t>
+          <t>11178935</t>
         </is>
       </c>
       <c r="D929" t="inlineStr">
         <is>
-          <t>Sp26Vac16Stan</t>
+          <t>SII26Tu10Gam</t>
         </is>
       </c>
       <c r="E929" t="inlineStr">
@@ -32911,17 +32911,17 @@
       </c>
       <c r="B930" s="7" t="inlineStr">
         <is>
-          <t>16918</t>
+          <t>16921</t>
         </is>
       </c>
       <c r="C930" s="7" t="inlineStr">
         <is>
-          <t>11178943</t>
+          <t>11178917</t>
         </is>
       </c>
       <c r="D930" t="inlineStr">
         <is>
-          <t>Sp26SS20Orange</t>
+          <t>WC26DW12Oran</t>
         </is>
       </c>
       <c r="E930" t="inlineStr">
@@ -32946,17 +32946,17 @@
       </c>
       <c r="B931" s="7" t="inlineStr">
         <is>
-          <t>16919</t>
+          <t>16923</t>
         </is>
       </c>
       <c r="C931" s="7" t="inlineStr">
         <is>
-          <t>11178957</t>
+          <t>11178918</t>
         </is>
       </c>
       <c r="D931" t="inlineStr">
         <is>
-          <t>WC26StanQuen30</t>
+          <t>WC26Gl20Silicone</t>
         </is>
       </c>
       <c r="E931" t="inlineStr">
@@ -32981,17 +32981,17 @@
       </c>
       <c r="B932" s="7" t="inlineStr">
         <is>
-          <t>16920</t>
+          <t>16924</t>
         </is>
       </c>
       <c r="C932" s="7" t="inlineStr">
         <is>
-          <t>11178935</t>
+          <t>11178945</t>
         </is>
       </c>
       <c r="D932" t="inlineStr">
         <is>
-          <t>SII26Tu10Gam</t>
+          <t>WC26Stan20IceF</t>
         </is>
       </c>
       <c r="E932" t="inlineStr">
@@ -33016,17 +33016,17 @@
       </c>
       <c r="B933" s="7" t="inlineStr">
         <is>
-          <t>16921</t>
+          <t>16925</t>
         </is>
       </c>
       <c r="C933" s="7" t="inlineStr">
         <is>
-          <t>11178917</t>
+          <t>11178973</t>
         </is>
       </c>
       <c r="D933" t="inlineStr">
         <is>
-          <t>WC26DW12Oran</t>
+          <t>WC26SS16Lid</t>
         </is>
       </c>
       <c r="E933" t="inlineStr">
@@ -33051,17 +33051,17 @@
       </c>
       <c r="B934" s="7" t="inlineStr">
         <is>
-          <t>16922</t>
+          <t>16958</t>
         </is>
       </c>
       <c r="C934" s="7" t="inlineStr">
         <is>
-          <t>11178919</t>
+          <t>11187370</t>
         </is>
       </c>
       <c r="D934" t="inlineStr">
         <is>
-          <t>Sp26Mug14Mom</t>
+          <t>WC26SS16Black</t>
         </is>
       </c>
       <c r="E934" t="inlineStr">
@@ -33086,17 +33086,17 @@
       </c>
       <c r="B935" s="7" t="inlineStr">
         <is>
-          <t>16923</t>
+          <t>16959</t>
         </is>
       </c>
       <c r="C935" s="7" t="inlineStr">
         <is>
-          <t>11178918</t>
+          <t>11187372</t>
         </is>
       </c>
       <c r="D935" t="inlineStr">
         <is>
-          <t>WC26Gl20Silicone</t>
+          <t>WC26Tu24DW</t>
         </is>
       </c>
       <c r="E935" t="inlineStr">
@@ -33121,17 +33121,13 @@
       </c>
       <c r="B936" s="7" t="inlineStr">
         <is>
-          <t>16924</t>
-        </is>
-      </c>
-      <c r="C936" s="7" t="inlineStr">
-        <is>
-          <t>11178945</t>
-        </is>
-      </c>
+          <t>16971</t>
+        </is>
+      </c>
+      <c r="C936" s="7" t="inlineStr"/>
       <c r="D936" t="inlineStr">
         <is>
-          <t>WC26Stan20IceF</t>
+          <t>WC26BearMex</t>
         </is>
       </c>
       <c r="E936" t="inlineStr">
@@ -33156,17 +33152,17 @@
       </c>
       <c r="B937" s="7" t="inlineStr">
         <is>
-          <t>16925</t>
+          <t>16978</t>
         </is>
       </c>
       <c r="C937" s="7" t="inlineStr">
         <is>
-          <t>11178973</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D937" t="inlineStr">
         <is>
-          <t>WC26SS16Lid</t>
+          <t>WC26LlaveroB</t>
         </is>
       </c>
       <c r="E937" t="inlineStr">
@@ -33186,12 +33182,12 @@
     <row r="938" ht="24" customHeight="1">
       <c r="A938" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B938" s="7" t="inlineStr">
         <is>
-          <t>16955</t>
+          <t>16531</t>
         </is>
       </c>
       <c r="C938" s="7" t="inlineStr">
@@ -33201,7 +33197,7 @@
       </c>
       <c r="D938" t="inlineStr">
         <is>
-          <t>WC26NESBX</t>
+          <t>Sp26NEBlack</t>
         </is>
       </c>
       <c r="E938" t="inlineStr">
@@ -33214,29 +33210,41 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="G938" t="inlineStr"/>
-      <c r="H938" t="inlineStr"/>
-      <c r="I938" t="inlineStr"/>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>lote-01/16531.jpeg</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I938" t="inlineStr">
+        <is>
+          <t>codigoDia</t>
+        </is>
+      </c>
     </row>
     <row r="939" ht="24" customHeight="1">
       <c r="A939" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B939" s="7" t="inlineStr">
         <is>
-          <t>16958</t>
+          <t>16532</t>
         </is>
       </c>
       <c r="C939" s="7" t="inlineStr">
         <is>
-          <t>11187370</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D939" t="inlineStr">
         <is>
-          <t>WC26SS16Black</t>
+          <t>Sp26NECrossB</t>
         </is>
       </c>
       <c r="E939" t="inlineStr">
@@ -33249,29 +33257,41 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="G939" t="inlineStr"/>
-      <c r="H939" t="inlineStr"/>
-      <c r="I939" t="inlineStr"/>
+      <c r="G939" t="inlineStr">
+        <is>
+          <t>lote-01/16532.jpeg</t>
+        </is>
+      </c>
+      <c r="H939" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I939" t="inlineStr">
+        <is>
+          <t>codigoDia</t>
+        </is>
+      </c>
     </row>
     <row r="940" ht="24" customHeight="1">
       <c r="A940" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B940" s="7" t="inlineStr">
         <is>
-          <t>16959</t>
+          <t>16601</t>
         </is>
       </c>
       <c r="C940" s="7" t="inlineStr">
         <is>
-          <t>11187372</t>
+          <t>11170187</t>
         </is>
       </c>
       <c r="D940" t="inlineStr">
         <is>
-          <t>WC26Tu24DW</t>
+          <t>ToteBag MxPais</t>
         </is>
       </c>
       <c r="E940" t="inlineStr">
@@ -33284,25 +33304,41 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="G940" t="inlineStr"/>
-      <c r="H940" t="inlineStr"/>
-      <c r="I940" t="inlineStr"/>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>lote-01/011170187.jpeg</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I940" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="941" ht="24" customHeight="1">
       <c r="A941" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B941" s="7" t="inlineStr">
         <is>
-          <t>16971</t>
-        </is>
-      </c>
-      <c r="C941" s="7" t="inlineStr"/>
+          <t>16643</t>
+        </is>
+      </c>
+      <c r="C941" s="7" t="inlineStr">
+        <is>
+          <t>11170102</t>
+        </is>
+      </c>
       <c r="D941" t="inlineStr">
         <is>
-          <t>WC26BearMex</t>
+          <t>DiscoveryCDMX</t>
         </is>
       </c>
       <c r="E941" t="inlineStr">
@@ -33315,29 +33351,41 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="G941" t="inlineStr"/>
-      <c r="H941" t="inlineStr"/>
-      <c r="I941" t="inlineStr"/>
+      <c r="G941" t="inlineStr">
+        <is>
+          <t>lote-01/011170102.jpeg</t>
+        </is>
+      </c>
+      <c r="H941" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I941" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="942" ht="24" customHeight="1">
       <c r="A942" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B942" s="7" t="inlineStr">
         <is>
-          <t>16978</t>
+          <t>16664</t>
         </is>
       </c>
       <c r="C942" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11176710</t>
         </is>
       </c>
       <c r="D942" t="inlineStr">
         <is>
-          <t>WC26LlaveroB</t>
+          <t>Sp26CC24Dome</t>
         </is>
       </c>
       <c r="E942" t="inlineStr">
@@ -33350,9 +33398,21 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="G942" t="inlineStr"/>
-      <c r="H942" t="inlineStr"/>
-      <c r="I942" t="inlineStr"/>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>lote-01/011176710.jpeg</t>
+        </is>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I942" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="943" ht="24" customHeight="1">
       <c r="A943" t="inlineStr">
@@ -33362,17 +33422,17 @@
       </c>
       <c r="B943" s="7" t="inlineStr">
         <is>
-          <t>16995</t>
+          <t>16681</t>
         </is>
       </c>
       <c r="C943" s="7" t="inlineStr">
         <is>
-          <t>11186650</t>
+          <t>11170174</t>
         </is>
       </c>
       <c r="D943" t="inlineStr">
         <is>
-          <t>SII26SS16Pleat</t>
+          <t>DiscCC24MxPais</t>
         </is>
       </c>
       <c r="E943" t="inlineStr">
@@ -33387,7 +33447,7 @@
       </c>
       <c r="G943" t="inlineStr">
         <is>
-          <t>lote-01/11186650.jpg</t>
+          <t>lote-01/011170174.jpeg</t>
         </is>
       </c>
       <c r="H943" t="inlineStr">
@@ -33409,17 +33469,17 @@
       </c>
       <c r="B944" s="7" t="inlineStr">
         <is>
-          <t>16997</t>
+          <t>16688</t>
         </is>
       </c>
       <c r="C944" s="7" t="inlineStr">
         <is>
-          <t>11186646</t>
+          <t>11170147</t>
         </is>
       </c>
       <c r="D944" t="inlineStr">
         <is>
-          <t>SII26SS12Charm</t>
+          <t>Disc2ozMxPais</t>
         </is>
       </c>
       <c r="E944" t="inlineStr">
@@ -33434,7 +33494,7 @@
       </c>
       <c r="G944" t="inlineStr">
         <is>
-          <t>lote-01/11186646.jpg</t>
+          <t>lote-01/011170147.jpeg</t>
         </is>
       </c>
       <c r="H944" t="inlineStr">
@@ -33456,17 +33516,17 @@
       </c>
       <c r="B945" s="7" t="inlineStr">
         <is>
-          <t>16998</t>
+          <t>16689</t>
         </is>
       </c>
       <c r="C945" s="7" t="inlineStr">
         <is>
-          <t>11186658</t>
+          <t>11170149</t>
         </is>
       </c>
       <c r="D945" t="inlineStr">
         <is>
-          <t>SII26SS20Hand</t>
+          <t>Disc2ozCDMX</t>
         </is>
       </c>
       <c r="E945" t="inlineStr">
@@ -33481,7 +33541,7 @@
       </c>
       <c r="G945" t="inlineStr">
         <is>
-          <t>lote-01/11186658.jpg</t>
+          <t>lote-01/011170149.jpeg</t>
         </is>
       </c>
       <c r="H945" t="inlineStr">
@@ -33503,17 +33563,17 @@
       </c>
       <c r="B946" s="7" t="inlineStr">
         <is>
-          <t>16999</t>
+          <t>16922</t>
         </is>
       </c>
       <c r="C946" s="7" t="inlineStr">
         <is>
-          <t>11186659</t>
+          <t>11178919</t>
         </is>
       </c>
       <c r="D946" t="inlineStr">
         <is>
-          <t>SII26BTLSS20</t>
+          <t>Sp26Mug14Mom</t>
         </is>
       </c>
       <c r="E946" t="inlineStr">
@@ -33528,7 +33588,7 @@
       </c>
       <c r="G946" t="inlineStr">
         <is>
-          <t>lote-01/11186659.jpg</t>
+          <t>lote-01/011178919.jpeg</t>
         </is>
       </c>
       <c r="H946" t="inlineStr">
@@ -33545,12 +33605,12 @@
     <row r="947" ht="24" customHeight="1">
       <c r="A947" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B947" s="7" t="inlineStr">
         <is>
-          <t>9616</t>
+          <t>16955</t>
         </is>
       </c>
       <c r="C947" s="7" t="inlineStr">
@@ -33560,7 +33620,7 @@
       </c>
       <c r="D947" t="inlineStr">
         <is>
-          <t>ESS Chemex 15oz</t>
+          <t>WC26NESBX</t>
         </is>
       </c>
       <c r="E947" t="inlineStr">
@@ -33570,32 +33630,44 @@
       </c>
       <c r="F947" t="inlineStr">
         <is>
-          <t>SECUNDARIO</t>
-        </is>
-      </c>
-      <c r="G947" t="inlineStr"/>
-      <c r="H947" t="inlineStr"/>
-      <c r="I947" t="inlineStr"/>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="G947" t="inlineStr">
+        <is>
+          <t>lote-01/16955.jpeg</t>
+        </is>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I947" t="inlineStr">
+        <is>
+          <t>codigoDia</t>
+        </is>
+      </c>
     </row>
     <row r="948" ht="24" customHeight="1">
       <c r="A948" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B948" s="7" t="inlineStr">
         <is>
-          <t>12480</t>
+          <t>16995</t>
         </is>
       </c>
       <c r="C948" s="7" t="inlineStr">
         <is>
-          <t>11103799</t>
+          <t>11186650</t>
         </is>
       </c>
       <c r="D948" t="inlineStr">
         <is>
-          <t>12480 Cafetera Green CJ/1 PZA</t>
+          <t>SII26SS16Pleat</t>
         </is>
       </c>
       <c r="E948" t="inlineStr">
@@ -33605,32 +33677,44 @@
       </c>
       <c r="F948" t="inlineStr">
         <is>
-          <t>SECUNDARIO</t>
-        </is>
-      </c>
-      <c r="G948" t="inlineStr"/>
-      <c r="H948" t="inlineStr"/>
-      <c r="I948" t="inlineStr"/>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>lote-01/11186650.jpg</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I948" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="949" ht="24" customHeight="1">
       <c r="A949" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B949" s="7" t="inlineStr">
         <is>
-          <t>12642</t>
+          <t>16997</t>
         </is>
       </c>
       <c r="C949" s="7" t="inlineStr">
         <is>
-          <t>11090466</t>
+          <t>11186646</t>
         </is>
       </c>
       <c r="D949" t="inlineStr">
         <is>
-          <t>CAFETERA BLACK TRITAN BEAKER 8TZ</t>
+          <t>SII26SS12Charm</t>
         </is>
       </c>
       <c r="E949" t="inlineStr">
@@ -33640,32 +33724,44 @@
       </c>
       <c r="F949" t="inlineStr">
         <is>
-          <t>SECUNDARIO</t>
-        </is>
-      </c>
-      <c r="G949" t="inlineStr"/>
-      <c r="H949" t="inlineStr"/>
-      <c r="I949" t="inlineStr"/>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="G949" t="inlineStr">
+        <is>
+          <t>lote-01/11186646.jpg</t>
+        </is>
+      </c>
+      <c r="H949" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I949" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="950" ht="24" customHeight="1">
       <c r="A950" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B950" s="7" t="inlineStr">
         <is>
-          <t>14779</t>
+          <t>16998</t>
         </is>
       </c>
       <c r="C950" s="7" t="inlineStr">
         <is>
-          <t>11129870</t>
+          <t>11186658</t>
         </is>
       </c>
       <c r="D950" t="inlineStr">
         <is>
-          <t>COR23 SSCC24 Sir</t>
+          <t>SII26SS20Hand</t>
         </is>
       </c>
       <c r="E950" t="inlineStr">
@@ -33675,32 +33771,44 @@
       </c>
       <c r="F950" t="inlineStr">
         <is>
-          <t>SECUNDARIO</t>
-        </is>
-      </c>
-      <c r="G950" t="inlineStr"/>
-      <c r="H950" t="inlineStr"/>
-      <c r="I950" t="inlineStr"/>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>lote-01/11186658.jpg</t>
+        </is>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I950" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="951" ht="24" customHeight="1">
       <c r="A951" t="inlineStr">
         <is>
-          <t>FALTA FOTO</t>
+          <t>CON FOTO</t>
         </is>
       </c>
       <c r="B951" s="7" t="inlineStr">
         <is>
-          <t>14780</t>
+          <t>16999</t>
         </is>
       </c>
       <c r="C951" s="7" t="inlineStr">
         <is>
-          <t>11129720</t>
+          <t>11186659</t>
         </is>
       </c>
       <c r="D951" t="inlineStr">
         <is>
-          <t>COR23 CC16 TinST</t>
+          <t>SII26BTLSS20</t>
         </is>
       </c>
       <c r="E951" t="inlineStr">
@@ -33710,12 +33818,24 @@
       </c>
       <c r="F951" t="inlineStr">
         <is>
-          <t>SECUNDARIO</t>
-        </is>
-      </c>
-      <c r="G951" t="inlineStr"/>
-      <c r="H951" t="inlineStr"/>
-      <c r="I951" t="inlineStr"/>
+          <t>ACTIVO</t>
+        </is>
+      </c>
+      <c r="G951" t="inlineStr">
+        <is>
+          <t>lote-01/11186659.jpg</t>
+        </is>
+      </c>
+      <c r="H951" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I951" t="inlineStr">
+        <is>
+          <t>skuIntl</t>
+        </is>
+      </c>
     </row>
     <row r="952" ht="24" customHeight="1">
       <c r="A952" t="inlineStr">
@@ -33725,17 +33845,17 @@
       </c>
       <c r="B952" s="7" t="inlineStr">
         <is>
-          <t>14781</t>
+          <t>9616</t>
         </is>
       </c>
       <c r="C952" s="7" t="inlineStr">
         <is>
-          <t>11129821</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D952" t="inlineStr">
         <is>
-          <t>COR23CC16 irid</t>
+          <t>ESS Chemex 15oz</t>
         </is>
       </c>
       <c r="E952" t="inlineStr">
@@ -33760,17 +33880,17 @@
       </c>
       <c r="B953" s="7" t="inlineStr">
         <is>
-          <t>14782</t>
+          <t>12480</t>
         </is>
       </c>
       <c r="C953" s="7" t="inlineStr">
         <is>
-          <t>11129797</t>
+          <t>11103799</t>
         </is>
       </c>
       <c r="D953" t="inlineStr">
         <is>
-          <t>COR23 CC16 Shell</t>
+          <t>12480 Cafetera Green CJ/1 PZA</t>
         </is>
       </c>
       <c r="E953" t="inlineStr">
@@ -33795,17 +33915,17 @@
       </c>
       <c r="B954" s="7" t="inlineStr">
         <is>
-          <t>14783</t>
+          <t>12642</t>
         </is>
       </c>
       <c r="C954" s="7" t="inlineStr">
         <is>
-          <t>11129846</t>
+          <t>11090466</t>
         </is>
       </c>
       <c r="D954" t="inlineStr">
         <is>
-          <t>COR23 KeyR TinST</t>
+          <t>CAFETERA BLACK TRITAN BEAKER 8TZ</t>
         </is>
       </c>
       <c r="E954" t="inlineStr">
@@ -33830,17 +33950,17 @@
       </c>
       <c r="B955" s="7" t="inlineStr">
         <is>
-          <t>14919</t>
+          <t>14779</t>
         </is>
       </c>
       <c r="C955" s="7" t="inlineStr">
         <is>
-          <t>11141068</t>
+          <t>11129870</t>
         </is>
       </c>
       <c r="D955" t="inlineStr">
         <is>
-          <t>COR23 Tu16 Siren</t>
+          <t>COR23 SSCC24 Sir</t>
         </is>
       </c>
       <c r="E955" t="inlineStr">
@@ -33865,17 +33985,17 @@
       </c>
       <c r="B956" s="7" t="inlineStr">
         <is>
-          <t>15996</t>
+          <t>14780</t>
         </is>
       </c>
       <c r="C956" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11129720</t>
         </is>
       </c>
       <c r="D956" t="inlineStr">
         <is>
-          <t>COR25CoffeeBean</t>
+          <t>COR23 CC16 TinST</t>
         </is>
       </c>
       <c r="E956" t="inlineStr">
@@ -33900,17 +34020,17 @@
       </c>
       <c r="B957" s="7" t="inlineStr">
         <is>
-          <t>16121</t>
+          <t>14781</t>
         </is>
       </c>
       <c r="C957" s="7" t="inlineStr">
         <is>
-          <t>11164269</t>
+          <t>11129821</t>
         </is>
       </c>
       <c r="D957" t="inlineStr">
         <is>
-          <t>SI25Tu16Charm</t>
+          <t>COR23CC16 irid</t>
         </is>
       </c>
       <c r="E957" t="inlineStr">
@@ -33935,17 +34055,17 @@
       </c>
       <c r="B958" s="7" t="inlineStr">
         <is>
-          <t>16127</t>
+          <t>14782</t>
         </is>
       </c>
       <c r="C958" s="7" t="inlineStr">
         <is>
-          <t>11164289</t>
+          <t>11129797</t>
         </is>
       </c>
       <c r="D958" t="inlineStr">
         <is>
-          <t>Fl25SSTu16B</t>
+          <t>COR23 CC16 Shell</t>
         </is>
       </c>
       <c r="E958" t="inlineStr">
@@ -33970,17 +34090,17 @@
       </c>
       <c r="B959" s="7" t="inlineStr">
         <is>
-          <t>16130</t>
+          <t>14783</t>
         </is>
       </c>
       <c r="C959" s="7" t="inlineStr">
         <is>
-          <t>11164299</t>
+          <t>11129846</t>
         </is>
       </c>
       <c r="D959" t="inlineStr">
         <is>
-          <t>SI25SS20Zoo</t>
+          <t>COR23 KeyR TinST</t>
         </is>
       </c>
       <c r="E959" t="inlineStr">
@@ -34005,17 +34125,17 @@
       </c>
       <c r="B960" s="7" t="inlineStr">
         <is>
-          <t>16148</t>
+          <t>14919</t>
         </is>
       </c>
       <c r="C960" s="7" t="inlineStr">
         <is>
-          <t>11164315</t>
+          <t>11141068</t>
         </is>
       </c>
       <c r="D960" t="inlineStr">
         <is>
-          <t>SII25Iceflow30</t>
+          <t>COR23 Tu16 Siren</t>
         </is>
       </c>
       <c r="E960" t="inlineStr">
@@ -34040,17 +34160,17 @@
       </c>
       <c r="B961" s="7" t="inlineStr">
         <is>
-          <t>16153</t>
+          <t>15996</t>
         </is>
       </c>
       <c r="C961" s="7" t="inlineStr">
         <is>
-          <t>11164278</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D961" t="inlineStr">
         <is>
-          <t>SI25BTL24Zoo</t>
+          <t>COR25CoffeeBean</t>
         </is>
       </c>
       <c r="E961" t="inlineStr">
@@ -34075,17 +34195,17 @@
       </c>
       <c r="B962" s="7" t="inlineStr">
         <is>
-          <t>16158</t>
+          <t>16121</t>
         </is>
       </c>
       <c r="C962" s="7" t="inlineStr">
         <is>
-          <t>11164260</t>
+          <t>11164269</t>
         </is>
       </c>
       <c r="D962" t="inlineStr">
         <is>
-          <t>Fl25Mug14Bar</t>
+          <t>SI25Tu16Charm</t>
         </is>
       </c>
       <c r="E962" t="inlineStr">
@@ -34110,17 +34230,17 @@
       </c>
       <c r="B963" s="7" t="inlineStr">
         <is>
-          <t>16159</t>
+          <t>16127</t>
         </is>
       </c>
       <c r="C963" s="7" t="inlineStr">
         <is>
-          <t>11164261</t>
+          <t>11164289</t>
         </is>
       </c>
       <c r="D963" t="inlineStr">
         <is>
-          <t>SI25Tz14Eleph</t>
+          <t>Fl25SSTu16B</t>
         </is>
       </c>
       <c r="E963" t="inlineStr">
@@ -34145,17 +34265,17 @@
       </c>
       <c r="B964" s="7" t="inlineStr">
         <is>
-          <t>16160</t>
+          <t>16130</t>
         </is>
       </c>
       <c r="C964" s="7" t="inlineStr">
         <is>
-          <t>11164262</t>
+          <t>11164299</t>
         </is>
       </c>
       <c r="D964" t="inlineStr">
         <is>
-          <t>SI25Mug14Mothers</t>
+          <t>SI25SS20Zoo</t>
         </is>
       </c>
       <c r="E964" t="inlineStr">
@@ -34180,17 +34300,17 @@
       </c>
       <c r="B965" s="7" t="inlineStr">
         <is>
-          <t>16161</t>
+          <t>16148</t>
         </is>
       </c>
       <c r="C965" s="7" t="inlineStr">
         <is>
-          <t>11164263</t>
+          <t>11164315</t>
         </is>
       </c>
       <c r="D965" t="inlineStr">
         <is>
-          <t>SI25DW12Mothers</t>
+          <t>SII25Iceflow30</t>
         </is>
       </c>
       <c r="E965" t="inlineStr">
@@ -34215,17 +34335,17 @@
       </c>
       <c r="B966" s="7" t="inlineStr">
         <is>
-          <t>16166</t>
+          <t>16153</t>
         </is>
       </c>
       <c r="C966" s="7" t="inlineStr">
         <is>
-          <t>11164291</t>
+          <t>11164278</t>
         </is>
       </c>
       <c r="D966" t="inlineStr">
         <is>
-          <t>SII25SS16Pearl</t>
+          <t>SI25BTL24Zoo</t>
         </is>
       </c>
       <c r="E966" t="inlineStr">
@@ -34250,17 +34370,17 @@
       </c>
       <c r="B967" s="7" t="inlineStr">
         <is>
-          <t>16167</t>
+          <t>16158</t>
         </is>
       </c>
       <c r="C967" s="7" t="inlineStr">
         <is>
-          <t>11164296</t>
+          <t>11164260</t>
         </is>
       </c>
       <c r="D967" t="inlineStr">
         <is>
-          <t>Fl25Tu20Silicon</t>
+          <t>Fl25Mug14Bar</t>
         </is>
       </c>
       <c r="E967" t="inlineStr">
@@ -34285,17 +34405,17 @@
       </c>
       <c r="B968" s="7" t="inlineStr">
         <is>
-          <t>16169</t>
+          <t>16159</t>
         </is>
       </c>
       <c r="C968" s="7" t="inlineStr">
         <is>
-          <t>11164301</t>
+          <t>11164261</t>
         </is>
       </c>
       <c r="D968" t="inlineStr">
         <is>
-          <t>SI25SSBTLZoo</t>
+          <t>SI25Tz14Eleph</t>
         </is>
       </c>
       <c r="E968" t="inlineStr">
@@ -34320,17 +34440,17 @@
       </c>
       <c r="B969" s="7" t="inlineStr">
         <is>
-          <t>16173</t>
+          <t>16160</t>
         </is>
       </c>
       <c r="C969" s="7" t="inlineStr">
         <is>
-          <t>11164308</t>
+          <t>11164262</t>
         </is>
       </c>
       <c r="D969" t="inlineStr">
         <is>
-          <t>SII25StanOrange</t>
+          <t>SI25Mug14Mothers</t>
         </is>
       </c>
       <c r="E969" t="inlineStr">
@@ -34355,17 +34475,17 @@
       </c>
       <c r="B970" s="7" t="inlineStr">
         <is>
-          <t>16177</t>
+          <t>16161</t>
         </is>
       </c>
       <c r="C970" s="7" t="inlineStr">
         <is>
-          <t>11164318</t>
+          <t>11164263</t>
         </is>
       </c>
       <c r="D970" t="inlineStr">
         <is>
-          <t>SII25KeyChain</t>
+          <t>SI25DW12Mothers</t>
         </is>
       </c>
       <c r="E970" t="inlineStr">
@@ -34390,17 +34510,17 @@
       </c>
       <c r="B971" s="7" t="inlineStr">
         <is>
-          <t>16181</t>
+          <t>16166</t>
         </is>
       </c>
       <c r="C971" s="7" t="inlineStr">
         <is>
-          <t>11167151</t>
+          <t>11164291</t>
         </is>
       </c>
       <c r="D971" t="inlineStr">
         <is>
-          <t>SII25CC24FRLenco</t>
+          <t>SII25SS16Pearl</t>
         </is>
       </c>
       <c r="E971" t="inlineStr">
@@ -34425,17 +34545,17 @@
       </c>
       <c r="B972" s="7" t="inlineStr">
         <is>
-          <t>16183</t>
+          <t>16167</t>
         </is>
       </c>
       <c r="C972" s="7" t="inlineStr">
         <is>
-          <t>11167153</t>
+          <t>11164296</t>
         </is>
       </c>
       <c r="D972" t="inlineStr">
         <is>
-          <t>SII25BTL20FarmR</t>
+          <t>Fl25Tu20Silicon</t>
         </is>
       </c>
       <c r="E972" t="inlineStr">
@@ -34460,17 +34580,17 @@
       </c>
       <c r="B973" s="7" t="inlineStr">
         <is>
-          <t>16184</t>
+          <t>16169</t>
         </is>
       </c>
       <c r="C973" s="7" t="inlineStr">
         <is>
-          <t>11167154</t>
+          <t>11164301</t>
         </is>
       </c>
       <c r="D973" t="inlineStr">
         <is>
-          <t>SII25Mug14FarmR</t>
+          <t>SI25SSBTLZoo</t>
         </is>
       </c>
       <c r="E973" t="inlineStr">
@@ -34495,17 +34615,17 @@
       </c>
       <c r="B974" s="7" t="inlineStr">
         <is>
-          <t>16225</t>
+          <t>16173</t>
         </is>
       </c>
       <c r="C974" s="7" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>11164308</t>
         </is>
       </c>
       <c r="D974" t="inlineStr">
         <is>
-          <t>Fl25ReusDDM</t>
+          <t>SII25StanOrange</t>
         </is>
       </c>
       <c r="E974" t="inlineStr">
@@ -34530,17 +34650,17 @@
       </c>
       <c r="B975" s="7" t="inlineStr">
         <is>
-          <t>16259</t>
+          <t>16177</t>
         </is>
       </c>
       <c r="C975" s="7" t="inlineStr">
         <is>
-          <t>11171525</t>
+          <t>11164318</t>
         </is>
       </c>
       <c r="D975" t="inlineStr">
         <is>
-          <t>SII25CCDomeBday</t>
+          <t>SII25KeyChain</t>
         </is>
       </c>
       <c r="E975" t="inlineStr">
@@ -34565,17 +34685,17 @@
       </c>
       <c r="B976" s="7" t="inlineStr">
         <is>
-          <t>16260</t>
+          <t>16181</t>
         </is>
       </c>
       <c r="C976" s="7" t="inlineStr">
         <is>
-          <t>11171526</t>
+          <t>11167151</t>
         </is>
       </c>
       <c r="D976" t="inlineStr">
         <is>
-          <t>SII25CCLlavero</t>
+          <t>SII25CC24FRLenco</t>
         </is>
       </c>
       <c r="E976" t="inlineStr">
@@ -34600,17 +34720,17 @@
       </c>
       <c r="B977" s="7" t="inlineStr">
         <is>
-          <t>16289</t>
+          <t>16183</t>
         </is>
       </c>
       <c r="C977" s="7" t="inlineStr">
         <is>
-          <t>11169485</t>
+          <t>11167153</t>
         </is>
       </c>
       <c r="D977" t="inlineStr">
         <is>
-          <t>Fl25PPFood</t>
+          <t>SII25BTL20FarmR</t>
         </is>
       </c>
       <c r="E977" t="inlineStr">
@@ -34635,17 +34755,17 @@
       </c>
       <c r="B978" s="7" t="inlineStr">
         <is>
-          <t>16314</t>
+          <t>16184</t>
         </is>
       </c>
       <c r="C978" s="7" t="inlineStr">
         <is>
-          <t>11169422</t>
+          <t>11167154</t>
         </is>
       </c>
       <c r="D978" t="inlineStr">
         <is>
-          <t>Fl25Mug14Bear</t>
+          <t>SII25Mug14FarmR</t>
         </is>
       </c>
       <c r="E978" t="inlineStr">
@@ -34670,17 +34790,17 @@
       </c>
       <c r="B979" s="7" t="inlineStr">
         <is>
-          <t>16316</t>
+          <t>16225</t>
         </is>
       </c>
       <c r="C979" s="7" t="inlineStr">
         <is>
-          <t>11169425</t>
+          <t>NA</t>
         </is>
       </c>
       <c r="D979" t="inlineStr">
         <is>
-          <t>Fl25Mug14Calav</t>
+          <t>Fl25ReusDDM</t>
         </is>
       </c>
       <c r="E979" t="inlineStr">
@@ -34705,17 +34825,17 @@
       </c>
       <c r="B980" s="7" t="inlineStr">
         <is>
-          <t>16324</t>
+          <t>16259</t>
         </is>
       </c>
       <c r="C980" s="7" t="inlineStr">
         <is>
-          <t>11169480</t>
+          <t>11171525</t>
         </is>
       </c>
       <c r="D980" t="inlineStr">
         <is>
-          <t>Fl25StanIceF</t>
+          <t>SII25CCDomeBday</t>
         </is>
       </c>
       <c r="E980" t="inlineStr">
@@ -34740,17 +34860,17 @@
       </c>
       <c r="B981" s="7" t="inlineStr">
         <is>
-          <t>16325</t>
+          <t>16260</t>
         </is>
       </c>
       <c r="C981" s="7" t="inlineStr">
         <is>
-          <t>11169484</t>
+          <t>11171526</t>
         </is>
       </c>
       <c r="D981" t="inlineStr">
         <is>
-          <t>Fl25CookieJar</t>
+          <t>SII25CCLlavero</t>
         </is>
       </c>
       <c r="E981" t="inlineStr">
@@ -34775,17 +34895,17 @@
       </c>
       <c r="B982" s="7" t="inlineStr">
         <is>
-          <t>16415</t>
+          <t>16289</t>
         </is>
       </c>
       <c r="C982" s="7" t="inlineStr">
         <is>
-          <t>Dinámica especial</t>
+          <t>11169485</t>
         </is>
       </c>
       <c r="D982" t="inlineStr">
         <is>
-          <t>SII25ReusPSL</t>
+          <t>Fl25PPFood</t>
         </is>
       </c>
       <c r="E982" t="inlineStr">
@@ -34810,17 +34930,17 @@
       </c>
       <c r="B983" s="7" t="inlineStr">
         <is>
-          <t>16434</t>
+          <t>16314</t>
         </is>
       </c>
       <c r="C983" s="7" t="inlineStr">
         <is>
-          <t>11173272</t>
+          <t>11169422</t>
         </is>
       </c>
       <c r="D983" t="inlineStr">
         <is>
-          <t>Xm25Tu12Lux</t>
+          <t>Fl25Mug14Bear</t>
         </is>
       </c>
       <c r="E983" t="inlineStr">
@@ -34845,17 +34965,17 @@
       </c>
       <c r="B984" s="7" t="inlineStr">
         <is>
-          <t>16460</t>
+          <t>16316</t>
         </is>
       </c>
       <c r="C984" s="7" t="inlineStr">
         <is>
-          <t>11172987</t>
+          <t>11169425</t>
         </is>
       </c>
       <c r="D984" t="inlineStr">
         <is>
-          <t>Xm25SS16Knit</t>
+          <t>Fl25Mug14Calav</t>
         </is>
       </c>
       <c r="E984" t="inlineStr">
@@ -34880,17 +35000,17 @@
       </c>
       <c r="B985" s="7" t="inlineStr">
         <is>
-          <t>16477</t>
+          <t>16324</t>
         </is>
       </c>
       <c r="C985" s="7" t="inlineStr">
         <is>
-          <t>11173043</t>
+          <t>11169480</t>
         </is>
       </c>
       <c r="D985" t="inlineStr">
         <is>
-          <t>Xm25GlassBear</t>
+          <t>Fl25StanIceF</t>
         </is>
       </c>
       <c r="E985" t="inlineStr">
@@ -34915,17 +35035,17 @@
       </c>
       <c r="B986" s="7" t="inlineStr">
         <is>
-          <t>16542</t>
+          <t>16325</t>
         </is>
       </c>
       <c r="C986" s="7" t="inlineStr">
         <is>
-          <t>11174790</t>
+          <t>11169484</t>
         </is>
       </c>
       <c r="D986" t="inlineStr">
         <is>
-          <t>Wt26Tu16Green</t>
+          <t>Fl25CookieJar</t>
         </is>
       </c>
       <c r="E986" t="inlineStr">
@@ -34950,17 +35070,17 @@
       </c>
       <c r="B987" s="7" t="inlineStr">
         <is>
-          <t>16668</t>
+          <t>16415</t>
         </is>
       </c>
       <c r="C987" s="7" t="inlineStr">
         <is>
-          <t>11176716</t>
+          <t>Dinámica especial</t>
         </is>
       </c>
       <c r="D987" t="inlineStr">
         <is>
-          <t>Sp26StanYellow20</t>
+          <t>SII25ReusPSL</t>
         </is>
       </c>
       <c r="E987" t="inlineStr">
@@ -34985,17 +35105,17 @@
       </c>
       <c r="B988" s="7" t="inlineStr">
         <is>
-          <t>16881</t>
+          <t>16434</t>
         </is>
       </c>
       <c r="C988" s="7" t="inlineStr">
         <is>
-          <t>11178933</t>
+          <t>11173272</t>
         </is>
       </c>
       <c r="D988" t="inlineStr">
         <is>
-          <t>SII25CC24Gamer</t>
+          <t>Xm25Tu12Lux</t>
         </is>
       </c>
       <c r="E988" t="inlineStr">
@@ -35020,13 +35140,17 @@
       </c>
       <c r="B989" s="7" t="inlineStr">
         <is>
-          <t>16977</t>
-        </is>
-      </c>
-      <c r="C989" s="7" t="inlineStr"/>
+          <t>16460</t>
+        </is>
+      </c>
+      <c r="C989" s="7" t="inlineStr">
+        <is>
+          <t>11172987</t>
+        </is>
+      </c>
       <c r="D989" t="inlineStr">
         <is>
-          <t>IMÁN MÉXICO</t>
+          <t>Xm25SS16Knit</t>
         </is>
       </c>
       <c r="E989" t="inlineStr">
@@ -35046,18 +35170,22 @@
     <row r="990" ht="24" customHeight="1">
       <c r="A990" t="inlineStr">
         <is>
-          <t>CON FOTO</t>
+          <t>FALTA FOTO</t>
         </is>
       </c>
       <c r="B990" s="7" t="inlineStr">
         <is>
-          <t>17359</t>
-        </is>
-      </c>
-      <c r="C990" s="7" t="inlineStr"/>
+          <t>16477</t>
+        </is>
+      </c>
+      <c r="C990" s="7" t="inlineStr">
+        <is>
+          <t>11173043</t>
+        </is>
+      </c>
       <c r="D990" t="inlineStr">
         <is>
-          <t>SII26GlCCColor</t>
+          <t>Xm25GlassBear</t>
         </is>
       </c>
       <c r="E990" t="inlineStr">
@@ -35070,37 +35198,29 @@
           <t>SECUNDARIO</t>
         </is>
       </c>
-      <c r="G990" t="inlineStr">
-        <is>
-          <t>lote-01/17359.jpg</t>
-        </is>
-      </c>
-      <c r="H990" t="inlineStr">
-        <is>
-          <t>lote-01</t>
-        </is>
-      </c>
-      <c r="I990" t="inlineStr">
-        <is>
-          <t>codigoDia</t>
-        </is>
-      </c>
+      <c r="G990" t="inlineStr"/>
+      <c r="H990" t="inlineStr"/>
+      <c r="I990" t="inlineStr"/>
     </row>
     <row r="991" ht="24" customHeight="1">
       <c r="A991" t="inlineStr">
         <is>
-          <t>CON FOTO</t>
+          <t>FALTA FOTO</t>
         </is>
       </c>
       <c r="B991" s="7" t="inlineStr">
         <is>
-          <t>17360</t>
-        </is>
-      </c>
-      <c r="C991" s="7" t="inlineStr"/>
+          <t>16542</t>
+        </is>
+      </c>
+      <c r="C991" s="7" t="inlineStr">
+        <is>
+          <t>11174790</t>
+        </is>
+      </c>
       <c r="D991" t="inlineStr">
         <is>
-          <t>SII26GlCCColor</t>
+          <t>Wt26Tu16Green</t>
         </is>
       </c>
       <c r="E991" t="inlineStr">
@@ -35113,72 +35233,247 @@
           <t>SECUNDARIO</t>
         </is>
       </c>
-      <c r="G991" t="inlineStr">
-        <is>
-          <t>lote-01/17360.jpg</t>
-        </is>
-      </c>
-      <c r="H991" t="inlineStr">
-        <is>
-          <t>lote-01</t>
-        </is>
-      </c>
-      <c r="I991" t="inlineStr">
-        <is>
-          <t>codigoDia</t>
-        </is>
-      </c>
+      <c r="G991" t="inlineStr"/>
+      <c r="H991" t="inlineStr"/>
+      <c r="I991" t="inlineStr"/>
     </row>
     <row r="992" ht="24" customHeight="1">
       <c r="A992" t="inlineStr">
         <is>
+          <t>FALTA FOTO</t>
+        </is>
+      </c>
+      <c r="B992" s="7" t="inlineStr">
+        <is>
+          <t>16668</t>
+        </is>
+      </c>
+      <c r="C992" s="7" t="inlineStr">
+        <is>
+          <t>11176716</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Sp26StanYellow20</t>
+        </is>
+      </c>
+      <c r="E992" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>SECUNDARIO</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr"/>
+      <c r="H992" t="inlineStr"/>
+      <c r="I992" t="inlineStr"/>
+    </row>
+    <row r="993" ht="24" customHeight="1">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>FALTA FOTO</t>
+        </is>
+      </c>
+      <c r="B993" s="7" t="inlineStr">
+        <is>
+          <t>16881</t>
+        </is>
+      </c>
+      <c r="C993" s="7" t="inlineStr">
+        <is>
+          <t>11178933</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>SII25CC24Gamer</t>
+        </is>
+      </c>
+      <c r="E993" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>SECUNDARIO</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr"/>
+      <c r="H993" t="inlineStr"/>
+      <c r="I993" t="inlineStr"/>
+    </row>
+    <row r="994" ht="24" customHeight="1">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>FALTA FOTO</t>
+        </is>
+      </c>
+      <c r="B994" s="7" t="inlineStr">
+        <is>
+          <t>16977</t>
+        </is>
+      </c>
+      <c r="C994" s="7" t="inlineStr"/>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>IMÁN MÉXICO</t>
+        </is>
+      </c>
+      <c r="E994" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>SECUNDARIO</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr"/>
+      <c r="H994" t="inlineStr"/>
+      <c r="I994" t="inlineStr"/>
+    </row>
+    <row r="995" ht="24" customHeight="1">
+      <c r="A995" t="inlineStr">
+        <is>
           <t>CON FOTO</t>
         </is>
       </c>
-      <c r="B992" s="7" t="inlineStr">
+      <c r="B995" s="7" t="inlineStr">
+        <is>
+          <t>17359</t>
+        </is>
+      </c>
+      <c r="C995" s="7" t="inlineStr"/>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>SII26GlCCColor</t>
+        </is>
+      </c>
+      <c r="E995" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>SECUNDARIO</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>lote-01/17359.jpg</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>codigoDia</t>
+        </is>
+      </c>
+    </row>
+    <row r="996" ht="24" customHeight="1">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>CON FOTO</t>
+        </is>
+      </c>
+      <c r="B996" s="7" t="inlineStr">
+        <is>
+          <t>17360</t>
+        </is>
+      </c>
+      <c r="C996" s="7" t="inlineStr"/>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>SII26GlCCColor</t>
+        </is>
+      </c>
+      <c r="E996" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>SECUNDARIO</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>lote-01/17360.jpg</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>lote-01</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>codigoDia</t>
+        </is>
+      </c>
+    </row>
+    <row r="997" ht="24" customHeight="1">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>CON FOTO</t>
+        </is>
+      </c>
+      <c r="B997" s="7" t="inlineStr">
         <is>
           <t>17362</t>
         </is>
       </c>
-      <c r="C992" s="7" t="inlineStr"/>
-      <c r="D992" t="inlineStr">
+      <c r="C997" s="7" t="inlineStr"/>
+      <c r="D997" t="inlineStr">
         <is>
           <t>SII26GlCCColor</t>
         </is>
       </c>
-      <c r="E992" t="inlineStr">
+      <c r="E997" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="F992" t="inlineStr">
+      <c r="F997" t="inlineStr">
         <is>
           <t>SECUNDARIO</t>
         </is>
       </c>
-      <c r="G992" t="inlineStr">
+      <c r="G997" t="inlineStr">
         <is>
           <t>lote-01/17362.jpg</t>
         </is>
       </c>
-      <c r="H992" t="inlineStr">
+      <c r="H997" t="inlineStr">
         <is>
           <t>lote-01</t>
         </is>
       </c>
-      <c r="I992" t="inlineStr">
+      <c r="I997" t="inlineStr">
         <is>
           <t>codigoDia</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:I992"/>
+  <autoFilter ref="A7:I997"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A6:I6"/>
   </mergeCells>
-  <conditionalFormatting sqref="A8:A992">
+  <conditionalFormatting sqref="A8:A997">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>A8="CON FOTO"</formula>
     </cfRule>

</xml_diff>